<commit_message>
v2: Two-pass scheduling, QA verification, draft/prod workflow, config-driven, multi-channel notifications
- Two-pass scheduling engine (initial fill + QA verification)
- Auto-fix violations and retry up to max_iterations
- Draft → Production workflow with identical sheet structure
- Comprehensive rules/configuration sheet with 6 sections
- Multi-channel notifications (Telegram, Email, WhatsApp)
- Auto change detection (checks draft 2x/day for manual edits)
- Configurable departments, shifts per day, people per shift
- v2 template with placeholder for 8 people, 2 departments, 5 weeks
</commit_message>
<xml_diff>
--- a/template/shifts_template.xlsx
+++ b/template/shifts_template.xlsx
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="8">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -48,10 +48,15 @@
     </font>
     <font>
       <b val="1"/>
-      <sz val="10"/>
+      <color rgb="002F5496"/>
+      <sz val="11"/>
     </font>
     <font>
       <sz val="9"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="10"/>
     </font>
   </fonts>
   <fills count="6">
@@ -104,7 +109,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
@@ -117,7 +122,9 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -127,10 +134,13 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -496,7 +506,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I31"/>
+  <dimension ref="A1:I34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -508,6 +518,12 @@
     <col width="14" customWidth="1" min="7" max="7"/>
     <col width="14" customWidth="1" min="8" max="8"/>
     <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="14" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -563,14 +579,14 @@
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>[צוות 1 - שם]</t>
+          <t>[מחלקה 1 - שם]</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>בוקר</t>
+          <t>משמרת 1</t>
         </is>
       </c>
       <c r="B4" s="6" t="n"/>
@@ -585,7 +601,7 @@
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>לילה</t>
+          <t>משמרת 2</t>
         </is>
       </c>
       <c r="B5" s="6" t="n"/>
@@ -600,7 +616,7 @@
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>[צוות 2 - שם]</t>
+          <t>[מחלקה 2 - שם]</t>
         </is>
       </c>
     </row>
@@ -650,7 +666,7 @@
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>בוקר</t>
+          <t>משמרת 1</t>
         </is>
       </c>
       <c r="B9" s="6" t="n"/>
@@ -665,7 +681,7 @@
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>לילה</t>
+          <t>משמרת 2</t>
         </is>
       </c>
       <c r="B10" s="6" t="n"/>
@@ -687,21 +703,21 @@
     <row r="13">
       <c r="A13" s="7" t="inlineStr">
         <is>
-          <t>1. החלף את [שם היחידה] בשם היחידה שלך</t>
+          <t>1. החלף/י את [שם היחידה] בשם היחידה</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="7" t="inlineStr">
         <is>
-          <t>2. החלף את [צוות 1 - שם] ו-[צוות 2 - שם] בשמות הצוותים</t>
+          <t>2. החלף/י את [מחלקה X - שם] בשמות המחלקות</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="7" t="inlineStr">
         <is>
-          <t>3. מלא/י את התאריכים בשורת התאריכים (שורה 2, 8)</t>
+          <t>3. מלא/י תאריכים בשורת הכותרות (7 ימים + עמודת סיכום ריקה)</t>
         </is>
       </c>
     </row>
@@ -712,6 +728,13 @@
         </is>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" s="7" t="inlineStr">
+        <is>
+          <t>5. הגדר/י את כללי התזמון בגיליון 'rules'</t>
+        </is>
+      </c>
+    </row>
     <row r="25">
       <c r="A25" s="8" t="inlineStr">
         <is>
@@ -727,42 +750,42 @@
       </c>
       <c r="B26" s="10" t="inlineStr">
         <is>
-          <t>עמודה 1</t>
+          <t>יום 1</t>
         </is>
       </c>
       <c r="C26" s="10" t="inlineStr">
         <is>
-          <t>עמודה 2</t>
+          <t>יום 2</t>
         </is>
       </c>
       <c r="D26" s="10" t="inlineStr">
         <is>
-          <t>עמודה 3</t>
+          <t>יום 3</t>
         </is>
       </c>
       <c r="E26" s="10" t="inlineStr">
         <is>
-          <t>עמודה 4</t>
+          <t>יום 4</t>
         </is>
       </c>
       <c r="F26" s="10" t="inlineStr">
         <is>
-          <t>עמודה 5</t>
+          <t>יום 5</t>
         </is>
       </c>
       <c r="G26" s="10" t="inlineStr">
         <is>
-          <t>עמודה 6</t>
+          <t>יום 6</t>
         </is>
       </c>
       <c r="H26" s="10" t="inlineStr">
         <is>
-          <t>עמודה 7</t>
+          <t>יום 7</t>
         </is>
       </c>
       <c r="I26" s="10" t="inlineStr">
         <is>
-          <t>עמודה 8</t>
+          <t>יום 8</t>
         </is>
       </c>
     </row>
@@ -996,6 +1019,147 @@
         </is>
       </c>
       <c r="I31" s="10" t="inlineStr">
+        <is>
+          <t>יכול</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="11" t="inlineStr">
+        <is>
+          <t>איש/אשת צוות 6</t>
+        </is>
+      </c>
+      <c r="B32" s="10" t="inlineStr">
+        <is>
+          <t>יכול</t>
+        </is>
+      </c>
+      <c r="C32" s="10" t="inlineStr">
+        <is>
+          <t>יכול</t>
+        </is>
+      </c>
+      <c r="D32" s="10" t="inlineStr">
+        <is>
+          <t>יכול</t>
+        </is>
+      </c>
+      <c r="E32" s="10" t="inlineStr">
+        <is>
+          <t>יכול</t>
+        </is>
+      </c>
+      <c r="F32" s="10" t="inlineStr">
+        <is>
+          <t>יכול</t>
+        </is>
+      </c>
+      <c r="G32" s="10" t="inlineStr">
+        <is>
+          <t>יכול</t>
+        </is>
+      </c>
+      <c r="H32" s="10" t="inlineStr">
+        <is>
+          <t>יכול</t>
+        </is>
+      </c>
+      <c r="I32" s="10" t="inlineStr">
+        <is>
+          <t>יכול</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="11" t="inlineStr">
+        <is>
+          <t>איש/אשת צוות 7</t>
+        </is>
+      </c>
+      <c r="B33" s="10" t="inlineStr">
+        <is>
+          <t>יכול</t>
+        </is>
+      </c>
+      <c r="C33" s="10" t="inlineStr">
+        <is>
+          <t>יכול</t>
+        </is>
+      </c>
+      <c r="D33" s="10" t="inlineStr">
+        <is>
+          <t>יכול</t>
+        </is>
+      </c>
+      <c r="E33" s="10" t="inlineStr">
+        <is>
+          <t>יכול</t>
+        </is>
+      </c>
+      <c r="F33" s="10" t="inlineStr">
+        <is>
+          <t>יכול</t>
+        </is>
+      </c>
+      <c r="G33" s="10" t="inlineStr">
+        <is>
+          <t>יכול</t>
+        </is>
+      </c>
+      <c r="H33" s="10" t="inlineStr">
+        <is>
+          <t>יכול</t>
+        </is>
+      </c>
+      <c r="I33" s="10" t="inlineStr">
+        <is>
+          <t>יכול</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="11" t="inlineStr">
+        <is>
+          <t>איש/אשת צוות 8</t>
+        </is>
+      </c>
+      <c r="B34" s="10" t="inlineStr">
+        <is>
+          <t>יכול</t>
+        </is>
+      </c>
+      <c r="C34" s="10" t="inlineStr">
+        <is>
+          <t>יכול</t>
+        </is>
+      </c>
+      <c r="D34" s="10" t="inlineStr">
+        <is>
+          <t>יכול</t>
+        </is>
+      </c>
+      <c r="E34" s="10" t="inlineStr">
+        <is>
+          <t>יכול</t>
+        </is>
+      </c>
+      <c r="F34" s="10" t="inlineStr">
+        <is>
+          <t>יכול</t>
+        </is>
+      </c>
+      <c r="G34" s="10" t="inlineStr">
+        <is>
+          <t>יכול</t>
+        </is>
+      </c>
+      <c r="H34" s="10" t="inlineStr">
+        <is>
+          <t>יכול</t>
+        </is>
+      </c>
+      <c r="I34" s="10" t="inlineStr">
         <is>
           <t>יכול</t>
         </is>
@@ -1018,19 +1182,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D17"/>
+  <dimension ref="A1:E56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="32" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="1" max="1"/>
     <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="45" customWidth="1" min="3" max="3"/>
-    <col width="40" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="55" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="12" t="inlineStr">
         <is>
-          <t>Scheduling Rules &amp; Configuration</t>
+          <t>Miluim Shift Scheduler — Configuration</t>
         </is>
       </c>
     </row>
@@ -1047,10 +1212,15 @@
       </c>
       <c r="C3" s="13" t="inlineStr">
         <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="D3" s="13" t="inlineStr">
+        <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="D3" s="13" t="inlineStr">
+      <c r="E3" s="13" t="inlineStr">
         <is>
           <t>Example</t>
         </is>
@@ -1059,302 +1229,1305 @@
     <row r="4">
       <c r="A4" s="14" t="inlineStr">
         <is>
-          <t>max_consecutive_nights</t>
-        </is>
-      </c>
-      <c r="B4" s="15" t="inlineStr">
+          <t># BASIC SCHEDULING</t>
+        </is>
+      </c>
+      <c r="B4" s="15" t="inlineStr"/>
+      <c r="C4" s="15" t="inlineStr">
+        <is>
+          <t>section</t>
+        </is>
+      </c>
+      <c r="D4" s="15" t="inlineStr"/>
+      <c r="E4" s="15" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="16" t="inlineStr">
+        <is>
+          <t>shifts_per_day</t>
+        </is>
+      </c>
+      <c r="B5" s="17" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="C4" s="15" t="inlineStr">
-        <is>
-          <t>Maximum consecutive night shifts per person</t>
-        </is>
-      </c>
-      <c r="D4" s="15" t="inlineStr">
+      <c r="C5" s="17" t="inlineStr">
+        <is>
+          <t>integer</t>
+        </is>
+      </c>
+      <c r="D5" s="17" t="inlineStr">
+        <is>
+          <t>Number of shifts per day</t>
+        </is>
+      </c>
+      <c r="E5" s="17" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="14" t="inlineStr">
-        <is>
-          <t>shift_times_morning</t>
-        </is>
-      </c>
-      <c r="B5" s="15" t="inlineStr">
+    <row r="6">
+      <c r="A6" s="16" t="inlineStr">
+        <is>
+          <t>shift_1_name</t>
+        </is>
+      </c>
+      <c r="B6" s="17" t="inlineStr">
+        <is>
+          <t>בוקר</t>
+        </is>
+      </c>
+      <c r="C6" s="17" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="D6" s="17" t="inlineStr">
+        <is>
+          <t>Name of first shift</t>
+        </is>
+      </c>
+      <c r="E6" s="17" t="inlineStr">
+        <is>
+          <t>בוקר (Morning)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="16" t="inlineStr">
+        <is>
+          <t>shift_2_name</t>
+        </is>
+      </c>
+      <c r="B7" s="17" t="inlineStr">
+        <is>
+          <t>לילה</t>
+        </is>
+      </c>
+      <c r="C7" s="17" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="D7" s="17" t="inlineStr">
+        <is>
+          <t>Name of second shift</t>
+        </is>
+      </c>
+      <c r="E7" s="17" t="inlineStr">
+        <is>
+          <t>לילה (Night)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="16" t="inlineStr">
+        <is>
+          <t>shift_1_hours</t>
+        </is>
+      </c>
+      <c r="B8" s="17" t="inlineStr">
         <is>
           <t>06:00-18:00</t>
         </is>
       </c>
-      <c r="C5" s="15" t="inlineStr">
-        <is>
-          <t>Morning shift time range</t>
-        </is>
-      </c>
-      <c r="D5" s="15" t="inlineStr">
+      <c r="C8" s="17" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="D8" s="17" t="inlineStr">
+        <is>
+          <t>Duration of first shift</t>
+        </is>
+      </c>
+      <c r="E8" s="17" t="inlineStr">
         <is>
           <t>06:00-18:00</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="14" t="inlineStr">
-        <is>
-          <t>shift_times_night</t>
-        </is>
-      </c>
-      <c r="B6" s="15" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="16" t="inlineStr">
+        <is>
+          <t>shift_2_hours</t>
+        </is>
+      </c>
+      <c r="B9" s="17" t="inlineStr">
         <is>
           <t>18:00-06:00</t>
         </is>
       </c>
-      <c r="C6" s="15" t="inlineStr">
-        <is>
-          <t>Night shift time range</t>
-        </is>
-      </c>
-      <c r="D6" s="15" t="inlineStr">
+      <c r="C9" s="17" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="D9" s="17" t="inlineStr">
+        <is>
+          <t>Duration of second shift</t>
+        </is>
+      </c>
+      <c r="E9" s="17" t="inlineStr">
         <is>
           <t>18:00-06:00</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="14" t="inlineStr">
-        <is>
-          <t>email_recipients</t>
-        </is>
-      </c>
-      <c r="B7" s="15" t="inlineStr"/>
-      <c r="C7" s="15" t="inlineStr">
-        <is>
-          <t>Comma-separated emails</t>
-        </is>
-      </c>
-      <c r="D7" s="15" t="inlineStr">
-        <is>
-          <t>a@b.com</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="14" t="inlineStr">
-        <is>
-          <t>date_start</t>
-        </is>
-      </c>
-      <c r="B8" s="15" t="inlineStr"/>
-      <c r="C8" s="15" t="inlineStr">
-        <is>
-          <t>First day (dd/mm/yyyy)</t>
-        </is>
-      </c>
-      <c r="D8" s="15" t="inlineStr">
-        <is>
-          <t>01/06/2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="14" t="inlineStr">
-        <is>
-          <t>date_end</t>
-        </is>
-      </c>
-      <c r="B9" s="15" t="inlineStr"/>
-      <c r="C9" s="15" t="inlineStr">
-        <is>
-          <t>Last day (dd/mm/yyyy)</t>
-        </is>
-      </c>
-      <c r="D9" s="15" t="inlineStr">
-        <is>
-          <t>08/07/2026</t>
-        </is>
-      </c>
-    </row>
     <row r="10">
-      <c r="A10" s="14" t="inlineStr">
-        <is>
-          <t>calendar_name</t>
-        </is>
-      </c>
-      <c r="B10" s="15" t="inlineStr">
-        <is>
-          <t>משמרות מילואים</t>
-        </is>
-      </c>
-      <c r="C10" s="15" t="inlineStr">
-        <is>
-          <t>Google Calendar name</t>
-        </is>
-      </c>
-      <c r="D10" s="15" t="inlineStr">
-        <is>
-          <t>משמרות מילואים</t>
+      <c r="A10" s="16" t="inlineStr">
+        <is>
+          <t>people_per_shift_1</t>
+        </is>
+      </c>
+      <c r="B10" s="17" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C10" s="17" t="inlineStr">
+        <is>
+          <t>integer</t>
+        </is>
+      </c>
+      <c r="D10" s="17" t="inlineStr">
+        <is>
+          <t>People needed per first shift slot</t>
+        </is>
+      </c>
+      <c r="E10" s="17" t="inlineStr">
+        <is>
+          <t>1</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="14" t="inlineStr">
-        <is>
-          <t>team_1_name</t>
-        </is>
-      </c>
-      <c r="B11" s="15" t="inlineStr">
-        <is>
-          <t>הערכה</t>
-        </is>
-      </c>
-      <c r="C11" s="15" t="inlineStr">
-        <is>
-          <t>Team 1 display name</t>
-        </is>
-      </c>
-      <c r="D11" s="15" t="inlineStr">
-        <is>
-          <t>הערכה</t>
+      <c r="A11" s="16" t="inlineStr">
+        <is>
+          <t>people_per_shift_2</t>
+        </is>
+      </c>
+      <c r="B11" s="17" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C11" s="17" t="inlineStr">
+        <is>
+          <t>integer</t>
+        </is>
+      </c>
+      <c r="D11" s="17" t="inlineStr">
+        <is>
+          <t>People needed per second shift slot</t>
+        </is>
+      </c>
+      <c r="E11" s="17" t="inlineStr">
+        <is>
+          <t>1</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="14" t="inlineStr">
         <is>
-          <t>team_2_name</t>
-        </is>
-      </c>
-      <c r="B12" s="15" t="inlineStr">
+          <t># DEPARTMENTS</t>
+        </is>
+      </c>
+      <c r="B12" s="15" t="inlineStr"/>
+      <c r="C12" s="15" t="inlineStr">
+        <is>
+          <t>section</t>
+        </is>
+      </c>
+      <c r="D12" s="15" t="inlineStr"/>
+      <c r="E12" s="15" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="16" t="inlineStr">
+        <is>
+          <t>num_departments</t>
+        </is>
+      </c>
+      <c r="B13" s="17" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C13" s="17" t="inlineStr">
+        <is>
+          <t>integer</t>
+        </is>
+      </c>
+      <c r="D13" s="17" t="inlineStr">
+        <is>
+          <t>Number of departments (e.g., הערכה, עיבוד)</t>
+        </is>
+      </c>
+      <c r="E13" s="17" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="16" t="inlineStr">
+        <is>
+          <t>department_1_name</t>
+        </is>
+      </c>
+      <c r="B14" s="17" t="inlineStr">
+        <is>
+          <t>הערכה</t>
+        </is>
+      </c>
+      <c r="C14" s="17" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="D14" s="17" t="inlineStr">
+        <is>
+          <t>Department 1 display name</t>
+        </is>
+      </c>
+      <c r="E14" s="17" t="inlineStr">
+        <is>
+          <t>הערכה</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="16" t="inlineStr">
+        <is>
+          <t>department_1_morning_row</t>
+        </is>
+      </c>
+      <c r="B15" s="17" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="C15" s="17" t="inlineStr">
+        <is>
+          <t>integer</t>
+        </is>
+      </c>
+      <c r="D15" s="17" t="inlineStr">
+        <is>
+          <t>Sheet row for dept 1 shift 1</t>
+        </is>
+      </c>
+      <c r="E15" s="17" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="16" t="inlineStr">
+        <is>
+          <t>department_1_night_row</t>
+        </is>
+      </c>
+      <c r="B16" s="17" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="C16" s="17" t="inlineStr">
+        <is>
+          <t>integer</t>
+        </is>
+      </c>
+      <c r="D16" s="17" t="inlineStr">
+        <is>
+          <t>Sheet row for dept 1 shift 2</t>
+        </is>
+      </c>
+      <c r="E16" s="17" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="16" t="inlineStr">
+        <is>
+          <t>department_2_name</t>
+        </is>
+      </c>
+      <c r="B17" s="17" t="inlineStr">
         <is>
           <t>עיבוד</t>
         </is>
       </c>
-      <c r="C12" s="15" t="inlineStr">
-        <is>
-          <t>Team 2 display name</t>
-        </is>
-      </c>
-      <c r="D12" s="15" t="inlineStr">
+      <c r="C17" s="17" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="D17" s="17" t="inlineStr">
+        <is>
+          <t>Department 2 display name</t>
+        </is>
+      </c>
+      <c r="E17" s="17" t="inlineStr">
         <is>
           <t>עיבוד</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="14" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="16" t="inlineStr">
+        <is>
+          <t>department_2_morning_row</t>
+        </is>
+      </c>
+      <c r="B18" s="17" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="C18" s="17" t="inlineStr">
+        <is>
+          <t>integer</t>
+        </is>
+      </c>
+      <c r="D18" s="17" t="inlineStr">
+        <is>
+          <t>Sheet row for dept 2 shift 1</t>
+        </is>
+      </c>
+      <c r="E18" s="17" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="16" t="inlineStr">
+        <is>
+          <t>department_2_night_row</t>
+        </is>
+      </c>
+      <c r="B19" s="17" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C19" s="17" t="inlineStr">
+        <is>
+          <t>integer</t>
+        </is>
+      </c>
+      <c r="D19" s="17" t="inlineStr">
+        <is>
+          <t>Sheet row for dept 2 shift 2</t>
+        </is>
+      </c>
+      <c r="E19" s="17" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="14" t="inlineStr">
+        <is>
+          <t># DATES</t>
+        </is>
+      </c>
+      <c r="B20" s="15" t="inlineStr"/>
+      <c r="C20" s="15" t="inlineStr">
+        <is>
+          <t>section</t>
+        </is>
+      </c>
+      <c r="D20" s="15" t="inlineStr"/>
+      <c r="E20" s="15" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="16" t="inlineStr">
+        <is>
+          <t>date_start</t>
+        </is>
+      </c>
+      <c r="B21" s="17" t="inlineStr"/>
+      <c r="C21" s="17" t="inlineStr">
+        <is>
+          <t>date</t>
+        </is>
+      </c>
+      <c r="D21" s="17" t="inlineStr">
+        <is>
+          <t>First scheduling day (dd/mm/yyyy)</t>
+        </is>
+      </c>
+      <c r="E21" s="17" t="inlineStr">
+        <is>
+          <t>01/06/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="16" t="inlineStr">
+        <is>
+          <t>date_end</t>
+        </is>
+      </c>
+      <c r="B22" s="17" t="inlineStr"/>
+      <c r="C22" s="17" t="inlineStr">
+        <is>
+          <t>date</t>
+        </is>
+      </c>
+      <c r="D22" s="17" t="inlineStr">
+        <is>
+          <t>Last scheduling day (dd/mm/yyyy)</t>
+        </is>
+      </c>
+      <c r="E22" s="17" t="inlineStr">
+        <is>
+          <t>08/07/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="14" t="inlineStr">
+        <is>
+          <t># SHEETS</t>
+        </is>
+      </c>
+      <c r="B23" s="15" t="inlineStr"/>
+      <c r="C23" s="15" t="inlineStr">
+        <is>
+          <t>section</t>
+        </is>
+      </c>
+      <c r="D23" s="15" t="inlineStr"/>
+      <c r="E23" s="15" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="16" t="inlineStr">
+        <is>
+          <t>draft_sheet_id</t>
+        </is>
+      </c>
+      <c r="B24" s="17" t="inlineStr"/>
+      <c r="C24" s="17" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="D24" s="17" t="inlineStr">
+        <is>
+          <t>Google Sheets ID of the DRAFT spreadsheet</t>
+        </is>
+      </c>
+      <c r="E24" s="17" t="inlineStr">
+        <is>
+          <t>1ABC...xyz</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="16" t="inlineStr">
+        <is>
+          <t>prod_sheet_id</t>
+        </is>
+      </c>
+      <c r="B25" s="17" t="inlineStr"/>
+      <c r="C25" s="17" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="D25" s="17" t="inlineStr">
+        <is>
+          <t>Google Sheets ID of the PRODUCTION spreadsheet</t>
+        </is>
+      </c>
+      <c r="E25" s="17" t="inlineStr">
+        <is>
+          <t>1DEF...uvw</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="16" t="inlineStr">
+        <is>
+          <t>draft_tab_name</t>
+        </is>
+      </c>
+      <c r="B26" s="17" t="inlineStr">
+        <is>
+          <t>משמרות</t>
+        </is>
+      </c>
+      <c r="C26" s="17" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="D26" s="17" t="inlineStr">
+        <is>
+          <t>Tab name for shifts in draft</t>
+        </is>
+      </c>
+      <c r="E26" s="17" t="inlineStr">
+        <is>
+          <t>משמרות</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="16" t="inlineStr">
+        <is>
+          <t>prod_tab_name</t>
+        </is>
+      </c>
+      <c r="B27" s="17" t="inlineStr">
+        <is>
+          <t>משמרות</t>
+        </is>
+      </c>
+      <c r="C27" s="17" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="D27" s="17" t="inlineStr">
+        <is>
+          <t>Tab name for shifts in production</t>
+        </is>
+      </c>
+      <c r="E27" s="17" t="inlineStr">
+        <is>
+          <t>משמרות</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="16" t="inlineStr">
         <is>
           <t>constraint_start_row</t>
         </is>
       </c>
-      <c r="B13" s="15" t="inlineStr">
+      <c r="B28" s="17" t="inlineStr">
         <is>
           <t>27</t>
         </is>
       </c>
-      <c r="C13" s="15" t="inlineStr">
-        <is>
-          <t>First row of constraints</t>
-        </is>
-      </c>
-      <c r="D13" s="15" t="inlineStr">
+      <c r="C28" s="17" t="inlineStr">
+        <is>
+          <t>integer</t>
+        </is>
+      </c>
+      <c r="D28" s="17" t="inlineStr">
+        <is>
+          <t>First row of constraint data</t>
+        </is>
+      </c>
+      <c r="E28" s="17" t="inlineStr">
         <is>
           <t>27</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="14" t="inlineStr">
+    <row r="29">
+      <c r="A29" s="16" t="inlineStr">
+        <is>
+          <t>constraint_name_column</t>
+        </is>
+      </c>
+      <c r="B29" s="17" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C29" s="17" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="D29" s="17" t="inlineStr">
+        <is>
+          <t>Column with person names in constraints</t>
+        </is>
+      </c>
+      <c r="E29" s="17" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="14" t="inlineStr">
+        <is>
+          <t># RULES</t>
+        </is>
+      </c>
+      <c r="B30" s="15" t="inlineStr"/>
+      <c r="C30" s="15" t="inlineStr">
+        <is>
+          <t>section</t>
+        </is>
+      </c>
+      <c r="D30" s="15" t="inlineStr"/>
+      <c r="E30" s="15" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="16" t="inlineStr">
+        <is>
+          <t>consecutive_night_limit</t>
+        </is>
+      </c>
+      <c r="B31" s="17" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C31" s="17" t="inlineStr">
+        <is>
+          <t>integer</t>
+        </is>
+      </c>
+      <c r="D31" s="17" t="inlineStr">
+        <is>
+          <t>Max consecutive night shifts per person (0=no limit)</t>
+        </is>
+      </c>
+      <c r="E31" s="17" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="16" t="inlineStr">
         <is>
           <t>rule_no_same_day</t>
         </is>
       </c>
-      <c r="B14" s="15" t="inlineStr">
+      <c r="B32" s="17" t="inlineStr">
         <is>
           <t>true</t>
         </is>
       </c>
-      <c r="C14" s="15" t="inlineStr">
-        <is>
-          <t>Prevent same person morning+night</t>
-        </is>
-      </c>
-      <c r="D14" s="15" t="inlineStr">
+      <c r="C32" s="17" t="inlineStr">
+        <is>
+          <t>boolean</t>
+        </is>
+      </c>
+      <c r="D32" s="17" t="inlineStr">
+        <is>
+          <t>Prevent same person on both shifts of one day</t>
+        </is>
+      </c>
+      <c r="E32" s="17" t="inlineStr">
         <is>
           <t>true</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="14" t="inlineStr">
+    <row r="33">
+      <c r="A33" s="16" t="inlineStr">
         <is>
           <t>rule_no_consecutive_night_morning</t>
         </is>
       </c>
-      <c r="B15" s="15" t="inlineStr">
+      <c r="B33" s="17" t="inlineStr">
         <is>
           <t>true</t>
         </is>
       </c>
-      <c r="C15" s="15" t="inlineStr">
-        <is>
-          <t>Prevent night-&gt;morning</t>
-        </is>
-      </c>
-      <c r="D15" s="15" t="inlineStr">
+      <c r="C33" s="17" t="inlineStr">
+        <is>
+          <t>boolean</t>
+        </is>
+      </c>
+      <c r="D33" s="17" t="inlineStr">
+        <is>
+          <t>Prevent night-&gt;morning consecutive</t>
+        </is>
+      </c>
+      <c r="E33" s="17" t="inlineStr">
         <is>
           <t>true</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="14" t="inlineStr">
+    <row r="34">
+      <c r="A34" s="16" t="inlineStr">
+        <is>
+          <t>rule_weekend_separation</t>
+        </is>
+      </c>
+      <c r="B34" s="17" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="C34" s="17" t="inlineStr">
+        <is>
+          <t>boolean</t>
+        </is>
+      </c>
+      <c r="D34" s="17" t="inlineStr">
+        <is>
+          <t>Try to avoid same person Fri+Sat</t>
+        </is>
+      </c>
+      <c r="E34" s="17" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="16" t="inlineStr">
+        <is>
+          <t>verification_enabled</t>
+        </is>
+      </c>
+      <c r="B35" s="17" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="C35" s="17" t="inlineStr">
+        <is>
+          <t>boolean</t>
+        </is>
+      </c>
+      <c r="D35" s="17" t="inlineStr">
+        <is>
+          <t>Run QA pass after initial scheduling</t>
+        </is>
+      </c>
+      <c r="E35" s="17" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="16" t="inlineStr">
+        <is>
+          <t>max_iterations</t>
+        </is>
+      </c>
+      <c r="B36" s="17" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C36" s="17" t="inlineStr">
+        <is>
+          <t>integer</t>
+        </is>
+      </c>
+      <c r="D36" s="17" t="inlineStr">
+        <is>
+          <t>Max scheduling iterations before alert</t>
+        </is>
+      </c>
+      <c r="E36" s="17" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="14" t="inlineStr">
+        <is>
+          <t># WORKFLOW</t>
+        </is>
+      </c>
+      <c r="B37" s="15" t="inlineStr"/>
+      <c r="C37" s="15" t="inlineStr">
+        <is>
+          <t>section</t>
+        </is>
+      </c>
+      <c r="D37" s="15" t="inlineStr"/>
+      <c r="E37" s="15" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="16" t="inlineStr">
+        <is>
+          <t>workflow_mode</t>
+        </is>
+      </c>
+      <c r="B38" s="17" t="inlineStr">
+        <is>
+          <t>draft_first</t>
+        </is>
+      </c>
+      <c r="C38" s="17" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="D38" s="17" t="inlineStr">
+        <is>
+          <t>draft_first | prod_direct | manual</t>
+        </is>
+      </c>
+      <c r="E38" s="17" t="inlineStr">
+        <is>
+          <t>draft_first</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="16" t="inlineStr">
+        <is>
+          <t>auto_verify_draft</t>
+        </is>
+      </c>
+      <c r="B39" s="17" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="C39" s="17" t="inlineStr">
+        <is>
+          <t>boolean</t>
+        </is>
+      </c>
+      <c r="D39" s="17" t="inlineStr">
+        <is>
+          <t>Auto-check draft for changes 2x/day</t>
+        </is>
+      </c>
+      <c r="E39" s="17" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="16" t="inlineStr">
+        <is>
+          <t>draft_check_times</t>
+        </is>
+      </c>
+      <c r="B40" s="17" t="inlineStr">
+        <is>
+          <t>09:00,15:00</t>
+        </is>
+      </c>
+      <c r="C40" s="17" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="D40" s="17" t="inlineStr">
+        <is>
+          <t>Times to check draft for changes</t>
+        </is>
+      </c>
+      <c r="E40" s="17" t="inlineStr">
+        <is>
+          <t>09:00,15:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="16" t="inlineStr">
+        <is>
+          <t>auto_copy_to_prod</t>
+        </is>
+      </c>
+      <c r="B41" s="17" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="C41" s="17" t="inlineStr">
+        <is>
+          <t>boolean</t>
+        </is>
+      </c>
+      <c r="D41" s="17" t="inlineStr">
+        <is>
+          <t>Auto-copy draft to prod after verification</t>
+        </is>
+      </c>
+      <c r="E41" s="17" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="14" t="inlineStr">
+        <is>
+          <t># NOTIFICATIONS</t>
+        </is>
+      </c>
+      <c r="B42" s="15" t="inlineStr"/>
+      <c r="C42" s="15" t="inlineStr">
+        <is>
+          <t>section</t>
+        </is>
+      </c>
+      <c r="D42" s="15" t="inlineStr"/>
+      <c r="E42" s="15" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="16" t="inlineStr">
+        <is>
+          <t>notify_channel_1</t>
+        </is>
+      </c>
+      <c r="B43" s="17" t="inlineStr">
+        <is>
+          <t>telegram</t>
+        </is>
+      </c>
+      <c r="C43" s="17" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="D43" s="17" t="inlineStr">
+        <is>
+          <t>Primary notification channel</t>
+        </is>
+      </c>
+      <c r="E43" s="17" t="inlineStr">
+        <is>
+          <t>telegram</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="16" t="inlineStr">
+        <is>
+          <t>notify_channel_2</t>
+        </is>
+      </c>
+      <c r="B44" s="17" t="inlineStr"/>
+      <c r="C44" s="17" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="D44" s="17" t="inlineStr">
+        <is>
+          <t>Secondary notification channel (email/whatsapp/telegram)</t>
+        </is>
+      </c>
+      <c r="E44" s="17" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="16" t="inlineStr">
+        <is>
+          <t>notify_channel_3</t>
+        </is>
+      </c>
+      <c r="B45" s="17" t="inlineStr"/>
+      <c r="C45" s="17" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="D45" s="17" t="inlineStr">
+        <is>
+          <t>Tertiary notification channel</t>
+        </is>
+      </c>
+      <c r="E45" s="17" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="16" t="inlineStr">
+        <is>
+          <t>telegram_chat_id</t>
+        </is>
+      </c>
+      <c r="B46" s="17" t="inlineStr"/>
+      <c r="C46" s="17" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="D46" s="17" t="inlineStr">
+        <is>
+          <t>Telegram chat ID for notifications</t>
+        </is>
+      </c>
+      <c r="E46" s="17" t="inlineStr">
+        <is>
+          <t>334721726</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="16" t="inlineStr">
+        <is>
+          <t>email_recipients</t>
+        </is>
+      </c>
+      <c r="B47" s="17" t="inlineStr"/>
+      <c r="C47" s="17" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="D47" s="17" t="inlineStr">
+        <is>
+          <t>Comma-separated email recipients</t>
+        </is>
+      </c>
+      <c r="E47" s="17" t="inlineStr">
+        <is>
+          <t>admin@unit.idf.il</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="16" t="inlineStr">
+        <is>
+          <t>notify_on_success</t>
+        </is>
+      </c>
+      <c r="B48" s="17" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="C48" s="17" t="inlineStr">
+        <is>
+          <t>boolean</t>
+        </is>
+      </c>
+      <c r="D48" s="17" t="inlineStr">
+        <is>
+          <t>Send notification when scheduling succeeds</t>
+        </is>
+      </c>
+      <c r="E48" s="17" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="16" t="inlineStr">
+        <is>
+          <t>notify_on_failure</t>
+        </is>
+      </c>
+      <c r="B49" s="17" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="C49" s="17" t="inlineStr">
+        <is>
+          <t>boolean</t>
+        </is>
+      </c>
+      <c r="D49" s="17" t="inlineStr">
+        <is>
+          <t>Send notification when scheduling fails</t>
+        </is>
+      </c>
+      <c r="E49" s="17" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="16" t="inlineStr">
+        <is>
+          <t>notify_on_draft_change</t>
+        </is>
+      </c>
+      <c r="B50" s="17" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="C50" s="17" t="inlineStr">
+        <is>
+          <t>boolean</t>
+        </is>
+      </c>
+      <c r="D50" s="17" t="inlineStr">
+        <is>
+          <t>Alert when draft sheet is modified</t>
+        </is>
+      </c>
+      <c r="E50" s="17" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="14" t="inlineStr">
+        <is>
+          <t># ADVANCED</t>
+        </is>
+      </c>
+      <c r="B51" s="15" t="inlineStr"/>
+      <c r="C51" s="15" t="inlineStr">
+        <is>
+          <t>section</t>
+        </is>
+      </c>
+      <c r="D51" s="15" t="inlineStr"/>
+      <c r="E51" s="15" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="16" t="inlineStr">
+        <is>
+          <t>calendar_name</t>
+        </is>
+      </c>
+      <c r="B52" s="17" t="inlineStr">
+        <is>
+          <t>משמרות מילואים</t>
+        </is>
+      </c>
+      <c r="C52" s="17" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="D52" s="17" t="inlineStr">
+        <is>
+          <t>Google Calendar display name</t>
+        </is>
+      </c>
+      <c r="E52" s="17" t="inlineStr">
+        <is>
+          <t>משמרות מילואים</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="16" t="inlineStr">
         <is>
           <t>report_send_time</t>
         </is>
       </c>
-      <c r="B16" s="15" t="inlineStr">
+      <c r="B53" s="17" t="inlineStr">
         <is>
           <t>07:00</t>
         </is>
       </c>
-      <c r="C16" s="15" t="inlineStr">
-        <is>
-          <t>Daily report time</t>
-        </is>
-      </c>
-      <c r="D16" s="15" t="inlineStr">
+      <c r="C53" s="17" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="D53" s="17" t="inlineStr">
+        <is>
+          <t>Time to send daily report email</t>
+        </is>
+      </c>
+      <c r="E53" s="17" t="inlineStr">
         <is>
           <t>07:00</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="14" t="inlineStr">
+    <row r="54">
+      <c r="A54" s="16" t="inlineStr">
         <is>
           <t>sync_time</t>
         </is>
       </c>
-      <c r="B17" s="15" t="inlineStr">
+      <c r="B54" s="17" t="inlineStr">
         <is>
           <t>06:30</t>
         </is>
       </c>
-      <c r="C17" s="15" t="inlineStr">
-        <is>
-          <t>Calendar sync time</t>
-        </is>
-      </c>
-      <c r="D17" s="15" t="inlineStr">
+      <c r="C54" s="17" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="D54" s="17" t="inlineStr">
+        <is>
+          <t>Time to sync with Google Calendar</t>
+        </is>
+      </c>
+      <c r="E54" s="17" t="inlineStr">
         <is>
           <t>06:30</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="16" t="inlineStr">
+        <is>
+          <t>date_cell_format</t>
+        </is>
+      </c>
+      <c r="B55" s="17" t="inlineStr">
+        <is>
+          <t>dd/mm/yy</t>
+        </is>
+      </c>
+      <c r="C55" s="17" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="D55" s="17" t="inlineStr">
+        <is>
+          <t>Date format used in headers</t>
+        </is>
+      </c>
+      <c r="E55" s="17" t="inlineStr">
+        <is>
+          <t>dd/mm/yy</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="16" t="inlineStr">
+        <is>
+          <t>summary_col_empty</t>
+        </is>
+      </c>
+      <c r="B56" s="17" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="C56" s="17" t="inlineStr">
+        <is>
+          <t>boolean</t>
+        </is>
+      </c>
+      <c r="D56" s="17" t="inlineStr">
+        <is>
+          <t>8th column of each week is summary (empty)</t>
+        </is>
+      </c>
+      <c r="E56" s="17" t="inlineStr">
+        <is>
+          <t>true</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A1:E1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1366,11 +2539,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D21"/>
+  <dimension ref="A1:D42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="50" customWidth="1" min="2" max="2"/>
+    <col width="35" customWidth="1" min="1" max="1"/>
+    <col width="65" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1381,192 +2554,380 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="16" t="inlineStr">
-        <is>
-          <t>How to Use</t>
-        </is>
-      </c>
-      <c r="B3" s="17" t="inlineStr"/>
+      <c r="A3" s="18" t="inlineStr">
+        <is>
+          <t>Quick Start</t>
+        </is>
+      </c>
+      <c r="B3" s="19" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" s="16" t="inlineStr">
-        <is>
-          <t>1. Fill in team names</t>
-        </is>
-      </c>
-      <c r="B4" s="17" t="inlineStr">
-        <is>
-          <t>Replace [name] placeholders in the 'משמרות' sheet</t>
+      <c r="A4" s="18" t="inlineStr">
+        <is>
+          <t>1. Duplicate this template twice</t>
+        </is>
+      </c>
+      <c r="B4" s="19" t="inlineStr">
+        <is>
+          <t>One is your DRAFT sheet, one is PRODUCTION</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="16" t="inlineStr">
-        <is>
-          <t>2. Set date headers</t>
-        </is>
-      </c>
-      <c r="B5" s="17" t="inlineStr">
-        <is>
-          <t>Add dates (7 days + 1 empty summary col per week)</t>
+      <c r="A5" s="18" t="inlineStr">
+        <is>
+          <t>2. Fill in your data</t>
+        </is>
+      </c>
+      <c r="B5" s="19" t="inlineStr">
+        <is>
+          <t>Names, constraints, dates</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="16" t="inlineStr">
-        <is>
-          <t>3. List your people</t>
-        </is>
-      </c>
-      <c r="B6" s="17" t="inlineStr">
-        <is>
-          <t>Replace 'איש/אשת צוות N' with real names in constraints</t>
+      <c r="A6" s="18" t="inlineStr">
+        <is>
+          <t>3. Configure the rules sheet</t>
+        </is>
+      </c>
+      <c r="B6" s="19" t="inlineStr">
+        <is>
+          <t>Set sheet IDs, shift config, notification channels</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="16" t="inlineStr">
-        <is>
-          <t>4. Set constraints</t>
-        </is>
-      </c>
-      <c r="B7" s="17" t="inlineStr">
-        <is>
-          <t>יכול | לא יכול | יכול רק בוקר | יכול רק לילה | לא ידוע</t>
+      <c r="A7" s="18" t="inlineStr">
+        <is>
+          <t>4. Run the scheduler</t>
+        </is>
+      </c>
+      <c r="B7" s="19" t="inlineStr">
+        <is>
+          <t>The agent does 2 passes: schedule + QA verification</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="16" t="inlineStr">
-        <is>
-          <t>5. Configure rules</t>
-        </is>
-      </c>
-      <c r="B8" s="17" t="inlineStr">
-        <is>
-          <t>Fill in the 'rules' sheet</t>
+      <c r="A8" s="18" t="inlineStr">
+        <is>
+          <t>5. Copy to production</t>
+        </is>
+      </c>
+      <c r="B8" s="19" t="inlineStr">
+        <is>
+          <t>After verification passes, copy draft → prod</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="16" t="inlineStr">
-        <is>
-          <t>6. Run the scheduler</t>
-        </is>
-      </c>
-      <c r="B9" s="17" t="inlineStr">
-        <is>
-          <t>Use the skill to generate the schedule</t>
-        </is>
-      </c>
+      <c r="A9" s="20" t="inlineStr"/>
+      <c r="B9" s="19" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" s="16" t="inlineStr"/>
-      <c r="B10" s="17" t="inlineStr"/>
+      <c r="A10" s="18" t="inlineStr">
+        <is>
+          <t>Two-Pass Scheduling</t>
+        </is>
+      </c>
+      <c r="B10" s="19" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" s="16" t="inlineStr">
+      <c r="A11" s="18" t="inlineStr">
+        <is>
+          <t>Pass 1: Initial Schedule</t>
+        </is>
+      </c>
+      <c r="B11" s="19" t="inlineStr">
+        <is>
+          <t>Greedy algorithm fills all shifts respecting constraints &amp; rules</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="18" t="inlineStr">
+        <is>
+          <t>Pass 2: QA Verification</t>
+        </is>
+      </c>
+      <c r="B12" s="19" t="inlineStr">
+        <is>
+          <t>Checks: same-day violations, rule2 violations, consecutive nights &gt; limit,</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="20" t="inlineStr"/>
+      <c r="B13" s="19" t="inlineStr">
+        <is>
+          <t>fairness variance, weekend separation, unassigned slots</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="20" t="inlineStr"/>
+      <c r="B14" s="19" t="inlineStr">
+        <is>
+          <t>If violations found: auto-fix and re-verify (up to max_iterations)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="20" t="inlineStr"/>
+      <c r="B15" s="19" t="inlineStr">
+        <is>
+          <t>On success: notify admin via configured channels</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="20" t="inlineStr"/>
+      <c r="B16" s="19" t="inlineStr">
+        <is>
+          <t>On failure after max iterations: alert admin with detailed report</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="20" t="inlineStr"/>
+      <c r="B17" s="19" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="18" t="inlineStr">
+        <is>
+          <t>Draft ↔ Production Workflow</t>
+        </is>
+      </c>
+      <c r="B18" s="19" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="18" t="inlineStr">
+        <is>
+          <t>Draft Sheet</t>
+        </is>
+      </c>
+      <c r="B19" s="19" t="inlineStr">
+        <is>
+          <t>Where the agent writes schedules. Can be edited manually.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="18" t="inlineStr">
+        <is>
+          <t>Production Sheet</t>
+        </is>
+      </c>
+      <c r="B20" s="19" t="inlineStr">
+        <is>
+          <t>The 'live' schedule used for calendar sync and reports.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="18" t="inlineStr">
+        <is>
+          <t>Copy Draft→Prod</t>
+        </is>
+      </c>
+      <c r="B21" s="19" t="inlineStr">
+        <is>
+          <t>Admin command: 'copy draft to prod'. Agent mirrors draft → prod.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="18" t="inlineStr">
+        <is>
+          <t>Auto-Check</t>
+        </is>
+      </c>
+      <c r="B22" s="19" t="inlineStr">
+        <is>
+          <t>Agent checks draft for manual changes 2x/day (configurable times)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="20" t="inlineStr"/>
+      <c r="B23" s="19" t="inlineStr">
+        <is>
+          <t>If draft changed: re-verify and notify admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="20" t="inlineStr"/>
+      <c r="B24" s="19" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="18" t="inlineStr">
         <is>
           <t>Constraint Legend</t>
         </is>
       </c>
-      <c r="B11" s="17" t="inlineStr"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="16" t="inlineStr">
-        <is>
-          <t>יכול</t>
-        </is>
-      </c>
-      <c r="B12" s="17" t="inlineStr">
-        <is>
-          <t>Available - can do any shift</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="16" t="inlineStr">
+      <c r="B25" s="19" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="18" t="inlineStr">
+        <is>
+          <t>יכול</t>
+        </is>
+      </c>
+      <c r="B26" s="19" t="inlineStr">
+        <is>
+          <t>Available — can do any shift</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="18" t="inlineStr">
         <is>
           <t>לא יכול</t>
         </is>
       </c>
-      <c r="B13" s="17" t="inlineStr">
-        <is>
-          <t>Not available</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="16" t="inlineStr">
+      <c r="B27" s="19" t="inlineStr">
+        <is>
+          <t>Not available — will not be assigned</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="18" t="inlineStr">
         <is>
           <t>יכול רק בוקר</t>
         </is>
       </c>
-      <c r="B14" s="17" t="inlineStr">
-        <is>
-          <t>Morning only</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="16" t="inlineStr">
+      <c r="B28" s="19" t="inlineStr">
+        <is>
+          <t>Shift 1 only — will only get first shift</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="18" t="inlineStr">
         <is>
           <t>יכול רק לילה</t>
         </is>
       </c>
-      <c r="B15" s="17" t="inlineStr">
-        <is>
-          <t>Night only</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="16" t="inlineStr">
+      <c r="B29" s="19" t="inlineStr">
+        <is>
+          <t>Shift 2 only — will only get second shift</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="18" t="inlineStr">
         <is>
           <t>לא ידוע</t>
         </is>
       </c>
-      <c r="B16" s="17" t="inlineStr">
-        <is>
-          <t>Unknown - treated as unavailable</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="16" t="inlineStr"/>
-      <c r="B17" s="17" t="inlineStr"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="16" t="inlineStr">
+      <c r="B30" s="19" t="inlineStr">
+        <is>
+          <t>Unknown — treated as unavailable (won't be assigned)</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="20" t="inlineStr"/>
+      <c r="B31" s="19" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="18" t="inlineStr">
+        <is>
+          <t>Notification Channels</t>
+        </is>
+      </c>
+      <c r="B32" s="19" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="18" t="inlineStr">
+        <is>
+          <t>telegram</t>
+        </is>
+      </c>
+      <c r="B33" s="19" t="inlineStr">
+        <is>
+          <t>Sends via configured Telegram bot</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="18" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="B34" s="19" t="inlineStr">
+        <is>
+          <t>Sends email to configured recipients</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="18" t="inlineStr">
+        <is>
+          <t>whatsapp</t>
+        </is>
+      </c>
+      <c r="B35" s="19" t="inlineStr">
+        <is>
+          <t>Sends via WhatsApp (requires integration)</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="20" t="inlineStr"/>
+      <c r="B36" s="19" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="18" t="inlineStr">
         <is>
           <t>Tips</t>
         </is>
       </c>
-      <c r="B18" s="17" t="inlineStr"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="16" t="inlineStr">
-        <is>
-          <t>• Summary columns (8th per week) stay empty for running totals</t>
-        </is>
-      </c>
-      <c r="B19" s="17" t="inlineStr"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="16" t="inlineStr">
-        <is>
-          <t>• The skill only fills future dates, never overwrites past</t>
-        </is>
-      </c>
-      <c r="B20" s="17" t="inlineStr"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="16" t="inlineStr">
-        <is>
-          <t>• Mark vacation days as 'לא יכול'</t>
-        </is>
-      </c>
-      <c r="B21" s="17" t="inlineStr"/>
+      <c r="B37" s="19" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="18" t="inlineStr">
+        <is>
+          <t>• Both draft and prod sheets must have IDENTICAL structure</t>
+        </is>
+      </c>
+      <c r="B38" s="19" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="18" t="inlineStr">
+        <is>
+          <t>• Summary columns (8th per week) stay empty — used for running totals</t>
+        </is>
+      </c>
+      <c r="B39" s="19" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="18" t="inlineStr">
+        <is>
+          <t>• The scheduler never overwrites past dates</t>
+        </is>
+      </c>
+      <c r="B40" s="19" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="18" t="inlineStr">
+        <is>
+          <t>• Mark vacation as 'לא יכול' for those days</t>
+        </is>
+      </c>
+      <c r="B41" s="19" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="18" t="inlineStr">
+        <is>
+          <t>• Verification checks: same-day, night→morning, consecutive limit, fairness, weekend</t>
+        </is>
+      </c>
+      <c r="B42" s="19" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
Add auto-publish option with admin approval fallback
auto_copy_to_prod: true = auto-publish draft to prod after QA passes
auto_copy_to_prod: false = notify admin, wait for copy-to-prod command
Both modes documented in SKILL.md, README.md and template rules sheet
</commit_message>
<xml_diff>
--- a/template/shifts_template.xlsx
+++ b/template/shifts_template.xlsx
@@ -2074,7 +2074,7 @@
       </c>
       <c r="D38" s="17" t="inlineStr">
         <is>
-          <t>draft_first | prod_direct | manual</t>
+          <t>draft_first = schedule in draft, then copy | prod_direct = write to prod | manual = no auto-scheduling</t>
         </is>
       </c>
       <c r="E38" s="17" t="inlineStr">
@@ -2155,7 +2155,7 @@
       </c>
       <c r="D41" s="17" t="inlineStr">
         <is>
-          <t>Auto-copy draft to prod after verification</t>
+          <t>true = auto-publish after QA passes | false = wait for admin approval</t>
         </is>
       </c>
       <c r="E41" s="17" t="inlineStr">

</xml_diff>

<commit_message>
Framework-agnostic: works with Claude Code, Hermes, OpenClaw. Team naming normalized.
- README: replaced 'Hermes' with 'AI agent', 'evaluation/analysis team' with 'team 1/team 2'
- SKILL.md: framework-agnostic docs, commands table per framework
- Template: normalized team references, 'framework-agnostic' in description
- Added rules config sheet to the actual Google Sheet with all settings
</commit_message>
<xml_diff>
--- a/template/shifts_template.xlsx
+++ b/template/shifts_template.xlsx
@@ -579,7 +579,7 @@
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>[מחלקה 1 - שם]</t>
+          <t>[Team 1 - שם]</t>
         </is>
       </c>
     </row>
@@ -613,10 +613,11 @@
       <c r="H5" s="6" t="n"/>
       <c r="I5" s="6" t="n"/>
     </row>
+    <row r="6"/>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>[מחלקה 2 - שם]</t>
+          <t>[Team 2 - שם]</t>
         </is>
       </c>
     </row>
@@ -693,6 +694,7 @@
       <c r="H10" s="6" t="n"/>
       <c r="I10" s="6" t="n"/>
     </row>
+    <row r="11"/>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
@@ -735,6 +737,13 @@
         </is>
       </c>
     </row>
+    <row r="18"/>
+    <row r="19"/>
+    <row r="20"/>
+    <row r="21"/>
+    <row r="22"/>
+    <row r="23"/>
+    <row r="24"/>
     <row r="25">
       <c r="A25" s="8" t="inlineStr">
         <is>
@@ -1199,6 +1208,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="13" t="inlineStr">
         <is>
@@ -1463,7 +1473,7 @@
       </c>
       <c r="D13" s="17" t="inlineStr">
         <is>
-          <t>Number of departments (e.g., הערכה, עיבוד)</t>
+          <t>Number of departments (e.g., Department 1, Department 2)</t>
         </is>
       </c>
       <c r="E13" s="17" t="inlineStr">
@@ -1480,7 +1490,7 @@
       </c>
       <c r="B14" s="17" t="inlineStr">
         <is>
-          <t>הערכה</t>
+          <t>Department 1</t>
         </is>
       </c>
       <c r="C14" s="17" t="inlineStr">
@@ -1495,7 +1505,7 @@
       </c>
       <c r="E14" s="17" t="inlineStr">
         <is>
-          <t>הערכה</t>
+          <t>Department 1</t>
         </is>
       </c>
     </row>
@@ -1561,7 +1571,7 @@
       </c>
       <c r="B17" s="17" t="inlineStr">
         <is>
-          <t>עיבוד</t>
+          <t>Department 2</t>
         </is>
       </c>
       <c r="C17" s="17" t="inlineStr">
@@ -1576,7 +1586,7 @@
       </c>
       <c r="E17" s="17" t="inlineStr">
         <is>
-          <t>עיבוד</t>
+          <t>Department 2</t>
         </is>
       </c>
     </row>
@@ -2553,6 +2563,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="18" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Rename rules sheet -> settings
</commit_message>
<xml_diff>
--- a/template/shifts_template.xlsx
+++ b/template/shifts_template.xlsx
@@ -8,7 +8,7 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="משמרות" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="rules" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="settings" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="instructions" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
@@ -613,7 +613,6 @@
       <c r="H5" s="6" t="n"/>
       <c r="I5" s="6" t="n"/>
     </row>
-    <row r="6"/>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
@@ -694,7 +693,6 @@
       <c r="H10" s="6" t="n"/>
       <c r="I10" s="6" t="n"/>
     </row>
-    <row r="11"/>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
@@ -737,13 +735,6 @@
         </is>
       </c>
     </row>
-    <row r="18"/>
-    <row r="19"/>
-    <row r="20"/>
-    <row r="21"/>
-    <row r="22"/>
-    <row r="23"/>
-    <row r="24"/>
     <row r="25">
       <c r="A25" s="8" t="inlineStr">
         <is>
@@ -1208,7 +1199,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="13" t="inlineStr">
         <is>
@@ -2563,7 +2553,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="18" t="inlineStr">
         <is>

</xml_diff>